<commit_message>
v9.4 — reset manuais + tooltip §3.8 + cálculo 100% automático
</commit_message>
<xml_diff>
--- a/Planilha_Mestre_Panorama_v9.4.xlsx
+++ b/Planilha_Mestre_Panorama_v9.4.xlsx
@@ -1333,7 +1333,7 @@
       </c>
       <c r="T9" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U9" s="12" t="inlineStr">
@@ -1557,11 +1557,11 @@
         <v>128250000</v>
       </c>
       <c r="S11" s="16" t="n">
-        <v>0.4526315789473684</v>
+        <v>0.4631578947368421</v>
       </c>
       <c r="T11" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U11" s="12" t="inlineStr">
@@ -2359,7 +2359,7 @@
       </c>
       <c r="T19" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U19" s="12" t="inlineStr">
@@ -2469,11 +2469,11 @@
         <v>141820500</v>
       </c>
       <c r="S20" s="10" t="n">
-        <v>0.833</v>
+        <v>0.8333333333333334</v>
       </c>
       <c r="T20" s="6" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U20" s="6" t="inlineStr">
@@ -2791,7 +2791,7 @@
       </c>
       <c r="T23" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U23" s="12" t="inlineStr">
@@ -2993,11 +2993,11 @@
         <v>106875000</v>
       </c>
       <c r="S25" s="16" t="n">
-        <v>0.736</v>
+        <v>0.752</v>
       </c>
       <c r="T25" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U25" s="12" t="inlineStr">
@@ -3216,12 +3216,10 @@
       <c r="R27" s="15" t="n">
         <v>87107197.5</v>
       </c>
-      <c r="S27" s="16" t="n">
-        <v>0.8666666666666667</v>
-      </c>
+      <c r="S27" s="16" t="n"/>
       <c r="T27" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="U27" s="12" t="inlineStr">
@@ -3330,12 +3328,10 @@
       <c r="R28" s="9" t="n">
         <v>91124130</v>
       </c>
-      <c r="S28" s="10" t="n">
-        <v>0.9166666666666666</v>
-      </c>
+      <c r="S28" s="10" t="n"/>
       <c r="T28" s="6" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="U28" s="6" t="inlineStr">
@@ -3445,11 +3441,11 @@
         <v>243300000</v>
       </c>
       <c r="S29" s="16" t="n">
-        <v>0.6919999999999999</v>
+        <v>0.6916666666666667</v>
       </c>
       <c r="T29" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U29" s="12" t="inlineStr">
@@ -3791,7 +3787,7 @@
       </c>
       <c r="T32" s="6" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U32" s="6" t="inlineStr">
@@ -4892,12 +4888,10 @@
       <c r="P43" s="15" t="n"/>
       <c r="Q43" s="15" t="n"/>
       <c r="R43" s="15" t="n"/>
-      <c r="S43" s="16" t="n">
-        <v>0.9399999999999999</v>
-      </c>
+      <c r="S43" s="16" t="n"/>
       <c r="T43" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="U43" s="12" t="inlineStr">
@@ -5103,7 +5097,7 @@
       </c>
       <c r="T45" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U45" s="12" t="inlineStr">
@@ -5312,12 +5306,10 @@
         <v>10796.46017699115</v>
       </c>
       <c r="R47" s="15" t="n"/>
-      <c r="S47" s="16" t="n">
-        <v>0.015625</v>
-      </c>
+      <c r="S47" s="16" t="n"/>
       <c r="T47" s="12" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="U47" s="12" t="inlineStr">
@@ -5431,7 +5423,7 @@
       </c>
       <c r="T48" s="6" t="inlineStr">
         <is>
-          <t>informado_manualmente</t>
+          <t>calculado_automatico</t>
         </is>
       </c>
       <c r="U48" s="6" t="inlineStr">

</xml_diff>